<commit_message>
Update scheme-saathi project.xlsx with new data
</commit_message>
<xml_diff>
--- a/teamProjectWorkspace/scheme-saathi project.xlsx
+++ b/teamProjectWorkspace/scheme-saathi project.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saurabhsrivastava/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Digvijay\IIT\CapstoneTeam\teamProjectWorkspace\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72675AA9-8E77-8942-A82C-D1457EBEF41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD78F34F-3C02-4C29-A279-DA82CF92C4E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="0" windowWidth="51200" windowHeight="21600" activeTab="1" xr2:uid="{7023AF24-8BA3-1E43-86F2-361958BC942A}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{7023AF24-8BA3-1E43-86F2-361958BC942A}"/>
   </bookViews>
   <sheets>
     <sheet name="Role &amp; Responsibility" sheetId="1" r:id="rId1"/>
@@ -28,8 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -37,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t>Role</t>
   </si>
@@ -277,13 +275,176 @@
   </si>
   <si>
     <t>Comment</t>
+  </si>
+  <si>
+    <r>
+      <t>Write a small function that turns a persona or household test case's </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Monaco"/>
+        <family val="2"/>
+      </rPr>
+      <t>profile_facts</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> into the rule fields (for example </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Monaco"/>
+        <family val="2"/>
+      </rPr>
+      <t>respondent_age</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Monaco"/>
+        <family val="2"/>
+      </rPr>
+      <t>age</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>). Add </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Monaco"/>
+        <family val="2"/>
+      </rPr>
+      <t>--persona-id</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Monaco"/>
+        <family val="2"/>
+      </rPr>
+      <t>graph.run</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> so a persona can be used instead of </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Monaco"/>
+        <family val="2"/>
+      </rPr>
+      <t>--citizen</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Digvijay</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Shows interest during the standup  meeting) - Persona-to-profile adapter - 29 Oct</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Digvijay</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="13"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Chat UI Interface for Chat Conversation</t>
+    </r>
+  </si>
+  <si>
+    <t>Inprogress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -324,6 +485,14 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -345,7 +514,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -356,6 +525,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -691,7 +863,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B022B9CE-43D1-7043-AC91-E98ECC06BB1D}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="34.1640625" customWidth="1"/>
     <col min="2" max="2" width="29.83203125" customWidth="1"/>
@@ -700,7 +872,7 @@
     <col min="5" max="5" width="41" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="16.5">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -714,7 +886,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="17">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -726,7 +898,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" ht="17">
       <c r="A3" s="1" t="s">
         <v>7</v>
       </c>
@@ -738,7 +910,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="17">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -750,7 +922,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="17">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -762,7 +934,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="17">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -774,7 +946,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" ht="17">
       <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
@@ -793,15 +965,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CAD46C4-7909-8F4B-9A9F-A24B8FE28E60}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="131.1640625" customWidth="1"/>
     <col min="2" max="2" width="35.6640625" customWidth="1"/>
     <col min="3" max="3" width="54.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3">
       <c r="A1" s="4" t="s">
         <v>30</v>
       </c>
@@ -812,42 +984,65 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="20" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="20">
       <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="17">
       <c r="A3" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="17">
       <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="17">
       <c r="A5" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="17">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="17">
       <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="17">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="83">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="17">
+      <c r="A11" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>